<commit_message>
Updated files with less number of accounts, beneficiaries and device counts
</commit_message>
<xml_diff>
--- a/outputs/Customer_Features_Catalogue.xlsx
+++ b/outputs/Customer_Features_Catalogue.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1088,6 +1088,94 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>shell_jurisdiction</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Incorporation jurisdiction for shell companies (BVI | Cayman | Panama | Delaware | Luxembourg | Seychelles | Mauritius | Singapore). NULL for non-shell beneficiaries. Secrecy jurisdictions = high AML risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>shell_age_days</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Days since shell company incorporation. NULL for non-shells. &lt;180 days = newly incorporated = highest risk for layering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ubo_disclosed</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1 = Ultimate Beneficial Owner identity is known. 0 = UBO hidden (red flag). NULL for non-shell beneficiaries. 75% of shells have hidden UBOs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>shell_newly_incorporated</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1 = shell company incorporated &lt;180 days ago. Strong layering risk signal. 0 for all non-shells and older shells.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding all output files
</commit_message>
<xml_diff>
--- a/outputs/Customer_Features_Catalogue.xlsx
+++ b/outputs/Customer_Features_Catalogue.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1088,6 +1088,94 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>shell_jurisdiction</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Incorporation jurisdiction for shell companies (BVI | Cayman | Panama | Delaware | Luxembourg | Seychelles | Mauritius | Singapore). NULL for non-shell beneficiaries. Secrecy jurisdictions = high AML risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>shell_age_days</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Days since shell company incorporation. NULL for non-shells. &lt;180 days = newly incorporated = highest risk for layering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ubo_disclosed</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1 = Ultimate Beneficial Owner identity is known. 0 = UBO hidden (red flag). NULL for non-shell beneficiaries. 75% of shells have hidden UBOs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>shell_newly_incorporated</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>beneficiaries</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1 = shell company incorporated &lt;180 days ago. Strong layering risk signal. 0 for all non-shells and older shells.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>